<commit_message>
Calendar v2: keep 3 posts a week, Reels replace project slots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mb6qwypygEVdYvV9LqQBFE
</commit_message>
<xml_diff>
--- a/social-media/VALDA_Content_Calendar_2026_v2.xlsx
+++ b/social-media/VALDA_Content_Calendar_2026_v2.xlsx
@@ -177,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,6 +219,7 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -584,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -592,12 +593,11 @@
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="58" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="52" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -610,7 +610,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A new blog article every 2 weeks (Monday) → carousel Tuesday → Reel Wednesday. Projects every other Friday; Behind the scenes on the others. Times ET; UK shown (clocks change UK 25 Oct, US 1 Nov).</t>
+          <t>Always 3 posts a week. Every 2 weeks: new blog on the website (Mon) → blog carousel (Tue) → product (Thu) → Reel on the blog topic (Fri, in place of a project). Other weeks: educational, product, project. Veterans Day (Wed 11 Nov) = Instagram Story only.</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Arm</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -663,11 +663,6 @@
       <c r="J4" s="15" t="inlineStr">
         <is>
           <t>Assets</t>
-        </is>
-      </c>
-      <c r="K4" s="15" t="inlineStr">
-        <is>
-          <t>Status</t>
         </is>
       </c>
     </row>
@@ -722,11 +717,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -775,11 +765,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -828,58 +813,44 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="K7" s="16" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>12 Oct</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr"/>
-      <c r="E8" s="17" t="inlineStr"/>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>BLOG</t>
-        </is>
-      </c>
-      <c r="G8" s="17" t="inlineStr">
-        <is>
-          <t>NEW article: What U-factor really tells you about a window</t>
-        </is>
-      </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr"/>
+      <c r="E8" s="23" t="inlineStr"/>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>BLOG (website only)</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>NEW article: What U-factor really tells you</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J8" s="17" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr"/>
+      <c r="J8" s="23" t="inlineStr">
         <is>
           <t>To write</t>
-        </is>
-      </c>
-      <c r="K8" s="17" t="inlineStr">
-        <is>
-          <t>Publish</t>
         </is>
       </c>
     </row>
@@ -916,7 +887,7 @@
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>U-factor (from the new article)</t>
+          <t>U-factor, from the new article</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
@@ -934,176 +905,152 @@
           <t>Expand from single</t>
         </is>
       </c>
-      <c r="K9" s="18" t="inlineStr">
-        <is>
-          <t>To build</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>14 Oct</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15 Oct</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>What we have</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Tilt and turn: one window, two ways to open</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Carousel (3)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>16 Oct</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="G10" s="19" t="inlineStr">
-        <is>
-          <t>U-factor Reel</t>
-        </is>
-      </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>U-factor Reel (replaces project)</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>Reel (12 s)</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="I11" s="19" t="inlineStr">
         <is>
           <t>https://valdagroup.com/insights/what-u-factor-tells-you</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
-      <c r="K10" s="19" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>15 Oct</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Tilt and turn: one window, two ways to open</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>20 Oct</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Educational</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Sightlines: more glass, less frame</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
         <is>
           <t>Built</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="F12" s="20" t="inlineStr">
-        <is>
-          <t>Behind the scenes</t>
-        </is>
-      </c>
-      <c r="G12" s="20" t="inlineStr">
-        <is>
-          <t>From Bulgaria to the USA</t>
-        </is>
-      </c>
-      <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>Carousel (7)</t>
-        </is>
-      </c>
-      <c r="I12" s="20" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/engineered-in-europe-delivered-worldwide</t>
-        </is>
-      </c>
-      <c r="J12" s="20" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K12" s="20" t="inlineStr">
-        <is>
-          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1115,32 +1062,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>20 Oct</t>
+          <t>22 Oct</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Educational</t>
+          <t>What we have</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Sightlines: more glass, less frame</t>
+          <t>Sliding and folding systems</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1154,221 +1101,192 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>22 Oct</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>23 Oct</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>American University of Malta</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>Photo + 2</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr"/>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>26 Oct</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr"/>
+      <c r="E15" s="23" t="inlineStr"/>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>BLOG (website only)</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>NEW article: The thermal break, explained</t>
+        </is>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr"/>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>To write</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>27 Oct</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Thermal break, from the new article</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Carousel (3)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>https://valdagroup.com/insights/thermal-break-explained</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>29 Oct</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>What we have</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Sliding and folding systems</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>The PVC range</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
         <is>
           <t>Built</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>23 Oct</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>Projects</t>
-        </is>
-      </c>
-      <c r="G15" s="16" t="inlineStr">
-        <is>
-          <t>American University of Malta</t>
-        </is>
-      </c>
-      <c r="H15" s="16" t="inlineStr">
-        <is>
-          <t>Photo + 2</t>
-        </is>
-      </c>
-      <c r="I15" s="16" t="inlineStr"/>
-      <c r="J15" s="16" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K15" s="16" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>26 Oct</t>
-        </is>
-      </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="D16" s="17" t="inlineStr"/>
-      <c r="E16" s="17" t="inlineStr"/>
-      <c r="F16" s="17" t="inlineStr">
-        <is>
-          <t>BLOG</t>
-        </is>
-      </c>
-      <c r="G16" s="17" t="inlineStr">
-        <is>
-          <t>NEW article: The thermal break, explained</t>
-        </is>
-      </c>
-      <c r="H16" s="17" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="I16" s="17" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J16" s="17" t="inlineStr">
-        <is>
-          <t>To write</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="inlineStr">
-        <is>
-          <t>Publish</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>27 Oct</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>1:00 PM</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="G17" s="18" t="inlineStr">
-        <is>
-          <t>Thermal break (from the new article)</t>
-        </is>
-      </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I17" s="18" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/thermal-break-explained</t>
-        </is>
-      </c>
-      <c r="J17" s="18" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K17" s="18" t="inlineStr">
-        <is>
-          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1380,22 +1298,22 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>28 Oct</t>
+          <t>30 Oct</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="F18" s="19" t="inlineStr">
@@ -1405,7 +1323,7 @@
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
-          <t>Thermal break Reel</t>
+          <t>Thermal break Reel (replaces project)</t>
         </is>
       </c>
       <c r="H18" s="19" t="inlineStr">
@@ -1421,53 +1339,48 @@
       <c r="J18" s="19" t="inlineStr">
         <is>
           <t>Built</t>
-        </is>
-      </c>
-      <c r="K18" s="19" t="inlineStr">
-        <is>
-          <t>Ready</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>29 Oct</t>
+          <t>03 Nov</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Tue</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>What we have</t>
+          <t>Educational</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The PVC range</t>
+          <t>Fixed or operable? Plan early</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Carousel (3)</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1476,396 +1389,348 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>30 Oct</t>
-        </is>
-      </c>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>05 Nov</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>What we have</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Facade systems: glazing at building scale</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Carousel (3)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>06 Nov</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Stella, Sofia</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Photo + 2</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr"/>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>09 Nov</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr"/>
+      <c r="E22" s="23" t="inlineStr"/>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>BLOG (website only)</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>NEW article: Triple glazing, when is it worth it?</t>
+        </is>
+      </c>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="inlineStr"/>
+      <c r="J22" s="23" t="inlineStr">
+        <is>
+          <t>To write</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>10 Nov</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>2:00 PM</t>
         </is>
       </c>
-      <c r="F20" s="20" t="inlineStr">
-        <is>
-          <t>Behind the scenes</t>
-        </is>
-      </c>
-      <c r="G20" s="20" t="inlineStr">
-        <is>
-          <t>How it works /01: a PVC profile</t>
-        </is>
-      </c>
-      <c r="H20" s="20" t="inlineStr">
-        <is>
-          <t>Reel (18 s)</t>
-        </is>
-      </c>
-      <c r="I20" s="20" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/how-pvc-window-profiles-are-made</t>
-        </is>
-      </c>
-      <c r="J20" s="20" t="inlineStr">
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>Triple glazing, from the new article</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>Carousel (3)</t>
+        </is>
+      </c>
+      <c r="I23" s="18" t="inlineStr">
+        <is>
+          <t>https://valdagroup.com/insights/is-triple-glazing-worth-it</t>
+        </is>
+      </c>
+      <c r="J23" s="18" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
-      <c r="K20" s="20" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>W5</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>03 Nov</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>12 Nov</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>What we have</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Dual-action windows, explained</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>13 Nov</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>Triple glazing Reel (replaces project)</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr"/>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> To make</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>17 Nov</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>2:00 PM</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Educational</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Fixed or operable? Plan early</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>What STC means for comfort</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Built</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>W5</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>05 Nov</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Facade systems: glazing at building scale</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>W5</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>06 Nov</t>
-        </is>
-      </c>
-      <c r="C23" s="16" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>Projects</t>
-        </is>
-      </c>
-      <c r="G23" s="16" t="inlineStr">
-        <is>
-          <t>Stella, Sofia</t>
-        </is>
-      </c>
-      <c r="H23" s="16" t="inlineStr">
-        <is>
-          <t>Photo + 2</t>
-        </is>
-      </c>
-      <c r="I23" s="16" t="inlineStr"/>
-      <c r="J23" s="16" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>09 Nov</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="D24" s="17" t="inlineStr"/>
-      <c r="E24" s="17" t="inlineStr"/>
-      <c r="F24" s="17" t="inlineStr">
-        <is>
-          <t>BLOG</t>
-        </is>
-      </c>
-      <c r="G24" s="17" t="inlineStr">
-        <is>
-          <t>NEW article: Triple glazing, when is it worth it?</t>
-        </is>
-      </c>
-      <c r="H24" s="17" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J24" s="17" t="inlineStr">
-        <is>
-          <t>To write</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>Publish</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>10 Nov</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="G25" s="18" t="inlineStr">
-        <is>
-          <t>Triple glazing (from the new article)</t>
-        </is>
-      </c>
-      <c r="H25" s="18" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I25" s="18" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/is-triple-glazing-worth-it</t>
-        </is>
-      </c>
-      <c r="J25" s="18" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K25" s="18" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>11 Nov</t>
-        </is>
-      </c>
-      <c r="C26" s="19" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E26" s="19" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>Reel + Holiday</t>
-        </is>
-      </c>
-      <c r="G26" s="19" t="inlineStr">
-        <is>
-          <t>Triple glazing Reel · Veterans Day as a Story / LinkedIn post</t>
-        </is>
-      </c>
-      <c r="H26" s="19" t="inlineStr">
-        <is>
-          <t>Reel + Story</t>
-        </is>
-      </c>
-      <c r="I26" s="19" t="inlineStr"/>
-      <c r="J26" s="19" t="inlineStr">
-        <is>
-          <t>Reel to make</t>
-        </is>
-      </c>
-      <c r="K26" s="19" t="inlineStr">
-        <is>
-          <t>To build</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>12 Nov</t>
+          <t>19 Nov</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1890,12 +1755,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Dual-action windows, explained</t>
+          <t>Casement systems: the classic, engineered</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Single</t>
+          <t>Carousel (3)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -1904,494 +1769,240 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="inlineStr">
-        <is>
-          <t>13 Nov</t>
-        </is>
-      </c>
-      <c r="C28" s="20" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>20 Nov</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="F28" s="20" t="inlineStr">
-        <is>
-          <t>Behind the scenes</t>
-        </is>
-      </c>
-      <c r="G28" s="20" t="inlineStr">
-        <is>
-          <t>How it works /03: US approval</t>
-        </is>
-      </c>
-      <c r="H28" s="20" t="inlineStr">
-        <is>
-          <t>Reel (20 s)</t>
-        </is>
-      </c>
-      <c r="I28" s="20" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/hvhz-vs-florida-product-approval</t>
-        </is>
-      </c>
-      <c r="J28" s="20" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>Juneau Village, Milwaukee (confirm building)</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>Photo + 2</t>
+        </is>
+      </c>
+      <c r="I28" s="16" t="inlineStr"/>
+      <c r="J28" s="16" t="inlineStr">
+        <is>
+          <t>Built, check</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>23 Nov</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr"/>
+      <c r="E29" s="23" t="inlineStr"/>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>BLOG (website only)</t>
+        </is>
+      </c>
+      <c r="G29" s="23" t="inlineStr">
+        <is>
+          <t>NEW article: How to read a window spec sheet</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="I29" s="23" t="inlineStr"/>
+      <c r="J29" s="23" t="inlineStr">
+        <is>
+          <t>To write</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>24 Nov</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="G30" s="18" t="inlineStr">
+        <is>
+          <t>How to read a spec sheet, from the new article</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>Carousel (5)</t>
+        </is>
+      </c>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>https://valdagroup.com/insights/how-to-read-a-window-spec-sheet</t>
+        </is>
+      </c>
+      <c r="J30" s="18" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
-      <c r="K28" s="20" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>17 Nov</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Educational</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>What STC means for comfort</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>26 Nov</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="E31" s="21" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="G31" s="21" t="inlineStr">
+        <is>
+          <t>Thanksgiving (replaces the product post)</t>
+        </is>
+      </c>
+      <c r="H31" s="21" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
+      <c r="I31" s="21" t="inlineStr"/>
+      <c r="J31" s="21" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>19 Nov</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Casement systems: the classic, engineered</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>20 Nov</t>
-        </is>
-      </c>
-      <c r="C31" s="16" t="inlineStr">
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>27 Nov</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="F31" s="16" t="inlineStr">
-        <is>
-          <t>Projects</t>
-        </is>
-      </c>
-      <c r="G31" s="16" t="inlineStr">
-        <is>
-          <t>Juneau Village, Milwaukee (confirm building)</t>
-        </is>
-      </c>
-      <c r="H31" s="16" t="inlineStr">
-        <is>
-          <t>Photo + 2</t>
-        </is>
-      </c>
-      <c r="I31" s="16" t="inlineStr"/>
-      <c r="J31" s="16" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K31" s="16" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>23 Nov</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="D32" s="17" t="inlineStr"/>
-      <c r="E32" s="17" t="inlineStr"/>
-      <c r="F32" s="17" t="inlineStr">
-        <is>
-          <t>BLOG</t>
-        </is>
-      </c>
-      <c r="G32" s="17" t="inlineStr">
-        <is>
-          <t>NEW article: How to read a window spec sheet</t>
-        </is>
-      </c>
-      <c r="H32" s="17" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="I32" s="17" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J32" s="17" t="inlineStr">
-        <is>
-          <t>To write</t>
-        </is>
-      </c>
-      <c r="K32" s="17" t="inlineStr">
-        <is>
-          <t>Publish</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B33" s="18" t="inlineStr">
-        <is>
-          <t>24 Nov</t>
-        </is>
-      </c>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="D33" s="18" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F33" s="18" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="G33" s="18" t="inlineStr">
-        <is>
-          <t>How to read a spec sheet (from the new article)</t>
-        </is>
-      </c>
-      <c r="H33" s="18" t="inlineStr">
-        <is>
-          <t>Carousel (5)</t>
-        </is>
-      </c>
-      <c r="I33" s="18" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/how-to-read-a-window-spec-sheet</t>
-        </is>
-      </c>
-      <c r="J33" s="18" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K33" s="18" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>25 Nov</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Glazing options, from double to triple (moved for Thanksgiving)</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="21" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B35" s="21" t="inlineStr">
-        <is>
-          <t>26 Nov</t>
-        </is>
-      </c>
-      <c r="C35" s="21" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D35" s="21" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E35" s="21" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="inlineStr">
-        <is>
-          <t>Holiday</t>
-        </is>
-      </c>
-      <c r="G35" s="21" t="inlineStr">
-        <is>
-          <t>Thanksgiving</t>
-        </is>
-      </c>
-      <c r="H35" s="21" t="inlineStr">
-        <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="I35" s="21" t="inlineStr"/>
-      <c r="J35" s="21" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K35" s="21" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="20" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B36" s="20" t="inlineStr">
-        <is>
-          <t>27 Nov</t>
-        </is>
-      </c>
-      <c r="C36" s="20" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D36" s="20" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="E36" s="20" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="F36" s="20" t="inlineStr">
-        <is>
-          <t>Behind the scenes</t>
-        </is>
-      </c>
-      <c r="G36" s="20" t="inlineStr">
-        <is>
-          <t>Myth vs fact /01: shutters</t>
-        </is>
-      </c>
-      <c r="H36" s="20" t="inlineStr">
-        <is>
-          <t>Reel (12 s)</t>
-        </is>
-      </c>
-      <c r="I36" s="20" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/impact-windows-vs-hurricane-shutters</t>
-        </is>
-      </c>
-      <c r="J36" s="20" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="K36" s="20" t="inlineStr">
-        <is>
-          <t>Ready</t>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>Spec sheet Reel: 5 numbers to check (replaces project)</t>
+        </is>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I32" s="19" t="inlineStr"/>
+      <c r="J32" s="19" t="inlineStr">
+        <is>
+          <t>To make</t>
         </is>
       </c>
     </row>
@@ -2598,8 +2209,6 @@
           <t>Content bank</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2622,8 +2231,6 @@
           <t>Content bank</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2646,8 +2253,6 @@
           <t>Content bank</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2670,8 +2275,6 @@
           <t>Content bank</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2684,11 +2287,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2702,11 +2305,6 @@
           <t>Why parked</t>
         </is>
       </c>
-      <c r="C1" s="22" t="inlineStr">
-        <is>
-          <t>Built?</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2719,11 +2317,6 @@
           <t>No architect or extra photos</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2733,12 +2326,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Architect unconfirmed (BLD MONA series)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Architect unconfirmed</t>
         </is>
       </c>
     </row>
@@ -2750,12 +2338,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Needs "the detail that mattered"; confirm phase</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Needs detail; confirm phase</t>
         </is>
       </c>
     </row>
@@ -2770,43 +2353,64 @@
           <t>No architect, one photo</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Reel: Hurricane impact test</t>
+          <t>Product: Glazing options, double to triple</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pair with HVHZ testing article in December</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Replaced by Thanksgiving</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Reel: How it works /02 shipping</t>
+          <t>Holiday: Veterans Day feed post</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pair with Engineered in Europe article</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Story only, to keep 3 posts a week</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carousel: From Bulgaria to the USA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Use in a December blog week (Engineered in Europe article)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Reel: How it works /01 PVC, /02 shipping, /03 US approval</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>December onward, paired with their articles</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Reel: Hurricane impact test, Myth vs fact /01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>December, paired with HVHZ and shutters articles</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Calendar v2: blended 4-week cycle of post types
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mb6qwypygEVdYvV9LqQBFE
</commit_message>
<xml_diff>
--- a/social-media/VALDA_Content_Calendar_2026_v2.xlsx
+++ b/social-media/VALDA_Content_Calendar_2026_v2.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Plan v2" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Blog schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Parked for later" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Original calendar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Content Bank" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Posting Guide" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cycle template" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Blog schedule" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Parked for later" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Original calendar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Content Bank" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Posting Guide" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -88,7 +89,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -150,6 +151,21 @@
         <fgColor rgb="00FDF5E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3EFE9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1ECF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -177,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -220,6 +236,9 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -585,32 +604,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>VALDA Content Calendar · Plan v2</t>
+          <t>VALDA Content Calendar · Plan v2 (blended)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Always 3 posts a week. Every 2 weeks: new blog on the website (Mon) → blog carousel (Tue) → product (Thu) → Reel on the blog topic (Fri, in place of a project). Other weeks: educational, product, project. Veterans Day (Wed 11 Nov) = Instagram Story only.</t>
+          <t>3 posts a week, rotating a 4-week cycle (A B C D). Per cycle: 3 product, 2 project, 2 blog, 2 Reel, 2 news, 1 educational. New blog goes live on the website on the Monday of B and D weeks.</t>
         </is>
       </c>
     </row>
@@ -622,24 +640,24 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Time (ET)</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>Time (UK)</t>
-        </is>
-      </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Type</t>
@@ -657,110 +675,99 @@
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>Links to</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
           <t>Assets</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>06 Oct</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>Educational</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Aluminium or PVC: how to choose</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>Carousel (5)</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/aluminum-vs-pvc-windows-hurricane</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="I5" s="24" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>08 Oct</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" s="25" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" s="25" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
         <is>
           <t>VALDA Vista: built to disappear</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>Carousel (5)</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
+      <c r="I6" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -774,27 +781,27 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
           <t>09 Oct</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>Projects</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
@@ -807,8 +814,7 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I7" s="16" t="inlineStr"/>
-      <c r="J7" s="16" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -822,33 +828,36 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
           <t>12 Oct</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr"/>
       <c r="E8" s="23" t="inlineStr"/>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>BLOG (website only)</t>
+          <t>(Website)</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>NEW article: What U-factor really tells you</t>
+          <t>NEW blog live: What U-factor really tells you</t>
         </is>
       </c>
       <c r="H8" s="23" t="inlineStr">
         <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="I8" s="23" t="inlineStr"/>
-      <c r="J8" s="23" t="inlineStr">
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -862,24 +871,24 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -897,206 +906,193 @@
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
-          <t>https://valdagroup.com/insights/what-u-factor-tells-you</t>
-        </is>
-      </c>
-      <c r="J9" s="18" t="inlineStr">
-        <is>
-          <t>Expand from single</t>
+          <t>Expand single</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>15 Oct</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>U-factor Reel</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Reel 12 s</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>16 Oct</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="G11" s="26" t="inlineStr">
+        <is>
+          <t>Company update: e.g. new US website live (confirm)</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>To make</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>20 Oct</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="F12" s="25" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="G12" s="25" t="inlineStr">
         <is>
           <t>Tilt and turn: one window, two ways to open</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H12" s="25" t="inlineStr">
         <is>
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
+      <c r="I12" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="F11" s="19" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>22 Oct</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="G11" s="19" t="inlineStr">
-        <is>
-          <t>U-factor Reel (replaces project)</t>
-        </is>
-      </c>
-      <c r="H11" s="19" t="inlineStr">
-        <is>
-          <t>Reel (12 s)</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/what-u-factor-tells-you</t>
-        </is>
-      </c>
-      <c r="J11" s="19" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>20 Oct</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Educational</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Sightlines: more glass, less frame</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>22 Oct</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Sliding and folding systems</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>How it works /01: a PVC profile</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Reel 18 s</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1110,27 +1106,27 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
           <t>23 Oct</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Projects</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
@@ -1143,8 +1139,7 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr"/>
-      <c r="J14" s="16" t="inlineStr">
+      <c r="I14" s="16" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1158,33 +1153,36 @@
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
           <t>26 Oct</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="D15" s="23" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="D15" s="23" t="inlineStr"/>
       <c r="E15" s="23" t="inlineStr"/>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>BLOG (website only)</t>
+          <t>(Website)</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
         <is>
-          <t>NEW article: The thermal break, explained</t>
+          <t>NEW blog live: The thermal break, explained</t>
         </is>
       </c>
       <c r="H15" s="23" t="inlineStr">
         <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="I15" s="23" t="inlineStr"/>
-      <c r="J15" s="23" t="inlineStr">
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -1198,24 +1196,24 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
           <t>27 Oct</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>1:00 PM</t>
-        </is>
-      </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1233,206 +1231,193 @@
       </c>
       <c r="I16" s="18" t="inlineStr">
         <is>
-          <t>https://valdagroup.com/insights/thermal-break-explained</t>
-        </is>
-      </c>
-      <c r="J16" s="18" t="inlineStr">
-        <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
         <is>
           <t>29 Oct</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" s="25" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" s="25" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>4:00 PM</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F17" s="25" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="G17" s="25" t="inlineStr">
         <is>
           <t>The PVC range</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="25" t="inlineStr">
         <is>
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
+      <c r="I17" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>30 Oct</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="D18" s="26" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>Thermal break Reel (replaces project)</t>
-        </is>
-      </c>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>Reel (15 s)</t>
-        </is>
-      </c>
-      <c r="I18" s="19" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/thermal-break-explained</t>
-        </is>
-      </c>
-      <c r="J18" s="19" t="inlineStr">
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="inlineStr">
+        <is>
+          <t>Behind the scenes: From Bulgaria to the USA</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>Carousel (7)</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>03 Nov</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="24" t="inlineStr">
         <is>
           <t>Educational</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Fixed or operable? Plan early</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>Sightlines: more glass, less frame</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
+        <is>
+          <t>Carousel (3)</t>
+        </is>
+      </c>
+      <c r="I19" s="24" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="inlineStr">
         <is>
           <t>05 Nov</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" s="25" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" s="25" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Facade systems: glazing at building scale</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="F20" s="25" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="G20" s="25" t="inlineStr">
+        <is>
+          <t>Sliding and folding systems</t>
+        </is>
+      </c>
+      <c r="H20" s="25" t="inlineStr">
         <is>
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
+      <c r="I20" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1446,27 +1431,27 @@
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
           <t>06 Nov</t>
         </is>
       </c>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>Projects</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
@@ -1479,8 +1464,7 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I21" s="16" t="inlineStr"/>
-      <c r="J21" s="16" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1494,33 +1478,36 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
           <t>09 Nov</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="D22" s="23" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr"/>
       <c r="E22" s="23" t="inlineStr"/>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>BLOG (website only)</t>
+          <t>(Website)</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>NEW article: Triple glazing, when is it worth it?</t>
+          <t>NEW blog live: Triple glazing, when is it worth it?</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
         <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="I22" s="23" t="inlineStr"/>
-      <c r="J22" s="23" t="inlineStr">
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -1534,24 +1521,24 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
           <t>10 Nov</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1569,202 +1556,193 @@
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>https://valdagroup.com/insights/is-triple-glazing-worth-it</t>
-        </is>
-      </c>
-      <c r="J23" s="18" t="inlineStr">
-        <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>12 Nov</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Dual-action windows, explained</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>Thermal break Reel</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Reel 15 s</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="B25" s="19" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
         <is>
           <t>13 Nov</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="D25" s="26" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E25" s="19" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
+      <c r="F25" s="26" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="G25" s="26" t="inlineStr">
+        <is>
+          <t>Inside the factory: our team and lines (photos needed)</t>
+        </is>
+      </c>
+      <c r="H25" s="26" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="I25" s="26" t="inlineStr">
+        <is>
+          <t>To make</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B26" s="25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>17 Nov</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E26" s="25" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="F26" s="25" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="G26" s="25" t="inlineStr">
+        <is>
+          <t>Facade systems: glazing at building scale</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>Carousel (3)</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>19 Nov</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="G25" s="19" t="inlineStr">
-        <is>
-          <t>Triple glazing Reel (replaces project)</t>
-        </is>
-      </c>
-      <c r="H25" s="19" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr"/>
-      <c r="J25" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> To make</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>17 Nov</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Educational</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>What STC means for comfort</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>19 Nov</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>What we have</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Casement systems: the classic, engineered</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Carousel (3)</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>How it works /03: US approval</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>Reel 20 s</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1778,27 +1756,27 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
           <t>20 Nov</t>
         </is>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
-          <t>Projects</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="G28" s="16" t="inlineStr">
@@ -1811,10 +1789,9 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I28" s="16" t="inlineStr"/>
-      <c r="J28" s="16" t="inlineStr">
-        <is>
-          <t>Built, check</t>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Built</t>
         </is>
       </c>
     </row>
@@ -1826,33 +1803,36 @@
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
           <t>23 Nov</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="D29" s="23" t="inlineStr"/>
       <c r="E29" s="23" t="inlineStr"/>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>BLOG (website only)</t>
+          <t>(Website)</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
         <is>
-          <t>NEW article: How to read a window spec sheet</t>
+          <t>NEW blog live: How to read a window spec sheet</t>
         </is>
       </c>
       <c r="H29" s="23" t="inlineStr">
         <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="I29" s="23" t="inlineStr"/>
-      <c r="J29" s="23" t="inlineStr">
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="I29" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -1866,24 +1846,24 @@
       </c>
       <c r="B30" s="18" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
           <t>24 Nov</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1900,11 +1880,6 @@
         </is>
       </c>
       <c r="I30" s="18" t="inlineStr">
-        <is>
-          <t>https://valdagroup.com/insights/how-to-read-a-window-spec-sheet</t>
-        </is>
-      </c>
-      <c r="J30" s="18" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1918,24 +1893,24 @@
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
           <t>26 Nov</t>
         </is>
       </c>
-      <c r="C31" s="21" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
       <c r="F31" s="21" t="inlineStr">
         <is>
           <t>Holiday</t>
@@ -1943,7 +1918,7 @@
       </c>
       <c r="G31" s="21" t="inlineStr">
         <is>
-          <t>Thanksgiving (replaces the product post)</t>
+          <t>Thanksgiving (takes the product slot)</t>
         </is>
       </c>
       <c r="H31" s="21" t="inlineStr">
@@ -1951,58 +1926,56 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="I31" s="21" t="inlineStr"/>
-      <c r="J31" s="21" t="inlineStr">
+      <c r="I31" s="21" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="B32" s="19" t="inlineStr">
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
         <is>
           <t>27 Nov</t>
         </is>
       </c>
-      <c r="C32" s="19" t="inlineStr">
+      <c r="D32" s="26" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="E32" s="26" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="F32" s="19" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="G32" s="19" t="inlineStr">
-        <is>
-          <t>Spec sheet Reel: 5 numbers to check (replaces project)</t>
-        </is>
-      </c>
-      <c r="H32" s="19" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="I32" s="19" t="inlineStr"/>
-      <c r="J32" s="19" t="inlineStr">
-        <is>
-          <t>To make</t>
+      <c r="F32" s="26" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="G32" s="26" t="inlineStr">
+        <is>
+          <t>Hurricane season ends 30 Nov: impact test Reel</t>
+        </is>
+      </c>
+      <c r="H32" s="26" t="inlineStr">
+        <is>
+          <t>Reel 15 s</t>
+        </is>
+      </c>
+      <c r="I32" s="26" t="inlineStr">
+        <is>
+          <t>Built</t>
         </is>
       </c>
     </row>
@@ -2012,6 +1985,148 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C1" s="22" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D1" s="22" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Educational</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B  (blog live Mon)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Blog carousel</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>News / update</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>D  (blog live Mon)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Blog carousel</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>News / update</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>News / update ideas</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Company news (website launch, new certification, trade show), behind the scenes, team, industry news (hurricane season, code changes)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2281,136 +2396,100 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="22" t="inlineStr">
-        <is>
-          <t>Why parked</t>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Project: Austin Residence</t>
+          <t>Educational: Fixed or operable</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>No architect or extra photos</t>
+          <t>Built; December</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Project: Mona Residence</t>
+          <t>Educational: What STC means</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Architect unconfirmed</t>
+          <t>Built; December</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Project: Amaya Residence</t>
+          <t>Product: Casement, Dual-action, Glazing options</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Needs detail; confirm phase</t>
+          <t>Built; December product slots</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Project: Belle Epoque</t>
+          <t>Projects: Austin, Mona, Amaya, Belle Epoque</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>No architect, one photo</t>
+          <t>Need photos and architects</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Product: Glazing options, double to triple</t>
+          <t>Reel: Myth vs fact /01, How it works /02 shipping</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Replaced by Thanksgiving</t>
+          <t>Built; December</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Holiday: Veterans Day feed post</t>
+          <t>Veterans Day (11 Nov)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Story only, to keep 3 posts a week</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Carousel: From Bulgaria to the USA</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Use in a December blog week (Engineered in Europe article)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Reel: How it works /01 PVC, /02 shipping, /03 US approval</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>December onward, paired with their articles</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Reel: Hurricane impact test, Myth vs fact /01</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>December, paired with HVHZ and shutters articles</t>
+          <t>Instagram Story only</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3763,7 +3842,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3979,7 +4058,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Calendar v2: add LinkedIn and Instagram format columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mb6qwypygEVdYvV9LqQBFE
</commit_message>
<xml_diff>
--- a/social-media/VALDA_Content_Calendar_2026_v2.xlsx
+++ b/social-media/VALDA_Content_Calendar_2026_v2.xlsx
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -615,7 +615,8 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -628,10 +629,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3 posts a week, rotating a 4-week cycle (A B C D). Per cycle: 3 product, 2 project, 2 blog, 2 Reel, 2 news, 1 educational. New blog goes live on the website on the Monday of B and D weeks.</t>
-        </is>
-      </c>
-    </row>
+          <t>3 posts a week, rotating a 4-week cycle (A B C D). Per cycle: 3 product, 2 project, 2 blog, 2 Reel, 2 news, 1 educational. New blog goes live on the website on the Monday of B and D weeks. Every post goes to LinkedIn (Buffer) and Instagram (Canva).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -675,6 +677,16 @@
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
           <t>Assets</t>
         </is>
       </c>
@@ -720,7 +732,17 @@
           <t>Carousel (5)</t>
         </is>
       </c>
-      <c r="I5" s="24" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Carousel 4:5</t>
+        </is>
+      </c>
+      <c r="K5" s="24" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -767,7 +789,17 @@
           <t>Carousel (5)</t>
         </is>
       </c>
-      <c r="I6" s="25" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Carousel 4:5</t>
+        </is>
+      </c>
+      <c r="K6" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -814,7 +846,17 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I7" s="16" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Carousel 4:5 + location + collab</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -857,7 +899,17 @@
           <t>Article</t>
         </is>
       </c>
-      <c r="I8" s="23" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Share the article link + LinkedIn newsletter / article version</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Link in bio updated</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -904,7 +956,17 @@
           <t>Carousel (5)</t>
         </is>
       </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>PDF carousel, article link in first comment</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Carousel 4:5, link in bio</t>
+        </is>
+      </c>
+      <c r="K9" s="18" t="inlineStr">
         <is>
           <t>Expand single</t>
         </is>
@@ -951,7 +1013,17 @@
           <t>Reel 12 s</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Native video</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Reel 9:16 + trending audio</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -998,7 +1070,17 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="I11" s="26" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Image or carousel post</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Carousel or Story</t>
+        </is>
+      </c>
+      <c r="K11" s="26" t="inlineStr">
         <is>
           <t>To make</t>
         </is>
@@ -1045,7 +1127,17 @@
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I12" s="25" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Carousel 4:5</t>
+        </is>
+      </c>
+      <c r="K12" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1092,7 +1184,17 @@
           <t>Reel 18 s</t>
         </is>
       </c>
-      <c r="I13" s="19" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Native video</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Reel 9:16 + trending audio</t>
+        </is>
+      </c>
+      <c r="K13" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1139,7 +1241,17 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Carousel 4:5 + location + collab</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1182,7 +1294,17 @@
           <t>Article</t>
         </is>
       </c>
-      <c r="I15" s="23" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Share the article link + LinkedIn newsletter / article version</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Link in bio updated</t>
+        </is>
+      </c>
+      <c r="K15" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -1229,7 +1351,17 @@
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I16" s="18" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>PDF carousel, article link in first comment</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Carousel 4:5, link in bio</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1276,7 +1408,17 @@
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I17" s="25" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Carousel 4:5</t>
+        </is>
+      </c>
+      <c r="K17" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1323,7 +1465,17 @@
           <t>Carousel (7)</t>
         </is>
       </c>
-      <c r="I18" s="26" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Image or carousel post</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Carousel or Story</t>
+        </is>
+      </c>
+      <c r="K18" s="26" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1370,7 +1522,17 @@
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I19" s="24" t="inlineStr">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Carousel 4:5</t>
+        </is>
+      </c>
+      <c r="K19" s="24" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1417,7 +1579,17 @@
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I20" s="25" t="inlineStr">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Carousel 4:5</t>
+        </is>
+      </c>
+      <c r="K20" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1464,7 +1636,17 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I21" s="16" t="inlineStr">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Carousel 4:5 + location + collab</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1507,7 +1689,17 @@
           <t>Article</t>
         </is>
       </c>
-      <c r="I22" s="23" t="inlineStr">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Share the article link + LinkedIn newsletter / article version</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Link in bio updated</t>
+        </is>
+      </c>
+      <c r="K22" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -1554,7 +1746,17 @@
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I23" s="18" t="inlineStr">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>PDF carousel, article link in first comment</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Carousel 4:5, link in bio</t>
+        </is>
+      </c>
+      <c r="K23" s="18" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1601,7 +1803,17 @@
           <t>Reel 15 s</t>
         </is>
       </c>
-      <c r="I24" s="19" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Native video</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Reel 9:16 + trending audio</t>
+        </is>
+      </c>
+      <c r="K24" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1648,7 +1860,17 @@
           <t>Carousel</t>
         </is>
       </c>
-      <c r="I25" s="26" t="inlineStr">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Image or carousel post</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Carousel or Story</t>
+        </is>
+      </c>
+      <c r="K25" s="26" t="inlineStr">
         <is>
           <t>To make</t>
         </is>
@@ -1695,7 +1917,17 @@
           <t>Carousel (3)</t>
         </is>
       </c>
-      <c r="I26" s="25" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Carousel 4:5</t>
+        </is>
+      </c>
+      <c r="K26" s="25" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1742,7 +1974,17 @@
           <t>Reel 20 s</t>
         </is>
       </c>
-      <c r="I27" s="19" t="inlineStr">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Native video</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Reel 9:16 + trending audio</t>
+        </is>
+      </c>
+      <c r="K27" s="19" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1789,7 +2031,17 @@
           <t>Photo + 2</t>
         </is>
       </c>
-      <c r="I28" s="16" t="inlineStr">
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>PDF carousel</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Carousel 4:5 + location + collab</t>
+        </is>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1832,7 +2084,17 @@
           <t>Article</t>
         </is>
       </c>
-      <c r="I29" s="23" t="inlineStr">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Share the article link + LinkedIn newsletter / article version</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Link in bio updated</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
         <is>
           <t>To write</t>
         </is>
@@ -1879,7 +2141,17 @@
           <t>Carousel (5)</t>
         </is>
       </c>
-      <c r="I30" s="18" t="inlineStr">
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>PDF carousel, article link in first comment</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Carousel 4:5, link in bio</t>
+        </is>
+      </c>
+      <c r="K30" s="18" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1926,7 +2198,17 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="I31" s="21" t="inlineStr">
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Image post</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Single image</t>
+        </is>
+      </c>
+      <c r="K31" s="21" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1973,7 +2255,17 @@
           <t>Reel 15 s</t>
         </is>
       </c>
-      <c r="I32" s="26" t="inlineStr">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Image or carousel post</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Carousel or Story</t>
+        </is>
+      </c>
+      <c r="K32" s="26" t="inlineStr">
         <is>
           <t>Built</t>
         </is>

</xml_diff>

<commit_message>
Document 2026 posting times, caption and hashtag rules; update the calendar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mb6qwypygEVdYvV9LqQBFE
</commit_message>
<xml_diff>
--- a/social-media/VALDA_Content_Calendar_2026_v2.xlsx
+++ b/social-media/VALDA_Content_Calendar_2026_v2.xlsx
@@ -629,11 +629,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3 posts a week, rotating a 4-week cycle (A B C D). Per cycle: 3 product, 2 project, 2 blog, 2 Reel, 2 news, 1 educational. New blog goes live on the website on the Monday of B and D weeks. Every post goes to LinkedIn (Buffer) and Instagram (Canva).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>3 posts a week. Projects every 3 weeks. New blog goes live on the website on alternate Mondays; the Tuesday after is the blog carousel. Times ET: LinkedIn Tue 10:00, Thu 11:00, Fri 10:00 · Instagram Tue/Thu 12:00, Fri 11:00, Reels 18:00. Every post goes to LinkedIn (Buffer) and Instagram (Canva).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Time ET (LI / IG)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -655,11 +661,7 @@
           <t>Day</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>Time (ET)</t>
-        </is>
-      </c>
+      <c r="E4" s="15" t="n"/>
       <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Type</t>
@@ -714,7 +716,7 @@
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F5" s="24" t="inlineStr">
@@ -724,7 +726,7 @@
       </c>
       <c r="G5" s="24" t="inlineStr">
         <is>
-          <t>Aluminium or PVC: how to choose</t>
+          <t>Aluminum or PVC: how to choose</t>
         </is>
       </c>
       <c r="H5" s="24" t="inlineStr">
@@ -744,7 +746,7 @@
       </c>
       <c r="K5" s="24" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -771,7 +773,7 @@
       </c>
       <c r="E6" s="25" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 12:00</t>
         </is>
       </c>
       <c r="F6" s="25" t="inlineStr">
@@ -781,7 +783,7 @@
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>VALDA Vista: built to disappear</t>
+          <t>VALDA Vista Guard</t>
         </is>
       </c>
       <c r="H6" s="25" t="inlineStr">
@@ -801,7 +803,7 @@
       </c>
       <c r="K6" s="25" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -828,7 +830,7 @@
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -858,7 +860,7 @@
       </c>
       <c r="K7" s="16" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -883,7 +885,11 @@
           <t>Mon</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr"/>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>9:00 (site)</t>
+        </is>
+      </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
           <t>(Website)</t>
@@ -891,7 +897,7 @@
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>NEW blog live: What U-factor really tells you</t>
+          <t>NEW article live: What U-factor really tells you</t>
         </is>
       </c>
       <c r="H8" s="23" t="inlineStr">
@@ -911,7 +917,7 @@
       </c>
       <c r="K8" s="23" t="inlineStr">
         <is>
-          <t>To write</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -938,7 +944,7 @@
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
@@ -968,7 +974,7 @@
       </c>
       <c r="K9" s="18" t="inlineStr">
         <is>
-          <t>Expand single</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -995,7 +1001,7 @@
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 18:00</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
@@ -1025,7 +1031,7 @@
       </c>
       <c r="K10" s="19" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1058,7 @@
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F11" s="26" t="inlineStr">
@@ -1062,12 +1068,12 @@
       </c>
       <c r="G11" s="26" t="inlineStr">
         <is>
-          <t>Company update: e.g. new US website live (confirm)</t>
+          <t>Meet VALDA: from a garage to two factories</t>
         </is>
       </c>
       <c r="H11" s="26" t="inlineStr">
         <is>
-          <t>Single</t>
+          <t>Carousel (5)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1082,7 +1088,7 @@
       </c>
       <c r="K11" s="26" t="inlineStr">
         <is>
-          <t>To make</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1115,7 @@
       </c>
       <c r="E12" s="25" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F12" s="25" t="inlineStr">
@@ -1119,7 +1125,7 @@
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>Tilt and turn: one window, two ways to open</t>
+          <t>Tilt and turn</t>
         </is>
       </c>
       <c r="H12" s="25" t="inlineStr">
@@ -1139,7 +1145,7 @@
       </c>
       <c r="K12" s="25" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1172,7 @@
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 18:00</t>
         </is>
       </c>
       <c r="F13" s="19" t="inlineStr">
@@ -1196,7 +1202,7 @@
       </c>
       <c r="K13" s="19" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1223,22 +1229,22 @@
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Behind the scenes</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>American University of Malta</t>
+          <t>From Bulgaria to the USA</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
         <is>
-          <t>Photo + 2</t>
+          <t>Carousel (7)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1253,7 +1259,7 @@
       </c>
       <c r="K14" s="16" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1284,11 @@
           <t>Mon</t>
         </is>
       </c>
-      <c r="E15" s="23" t="inlineStr"/>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>9:00 (site)</t>
+        </is>
+      </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
           <t>(Website)</t>
@@ -1286,7 +1296,7 @@
       </c>
       <c r="G15" s="23" t="inlineStr">
         <is>
-          <t>NEW blog live: The thermal break, explained</t>
+          <t>NEW article live: The thermal break, explained</t>
         </is>
       </c>
       <c r="H15" s="23" t="inlineStr">
@@ -1306,7 +1316,7 @@
       </c>
       <c r="K15" s="23" t="inlineStr">
         <is>
-          <t>To write</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1343,7 @@
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
@@ -1363,7 +1373,7 @@
       </c>
       <c r="K16" s="18" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1400,7 @@
       </c>
       <c r="E17" s="25" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 12:00</t>
         </is>
       </c>
       <c r="F17" s="25" t="inlineStr">
@@ -1420,7 +1430,7 @@
       </c>
       <c r="K17" s="25" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1447,22 +1457,22 @@
       </c>
       <c r="E18" s="26" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="G18" s="26" t="inlineStr">
         <is>
-          <t>Behind the scenes: From Bulgaria to the USA</t>
+          <t>American University of Malta</t>
         </is>
       </c>
       <c r="H18" s="26" t="inlineStr">
         <is>
-          <t>Carousel (7)</t>
+          <t>Photo + 2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1477,7 +1487,7 @@
       </c>
       <c r="K18" s="26" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Built, awaiting approval</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1514,7 @@
       </c>
       <c r="E19" s="24" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F19" s="24" t="inlineStr">
@@ -1514,7 +1524,7 @@
       </c>
       <c r="G19" s="24" t="inlineStr">
         <is>
-          <t>Sightlines: more glass, less frame</t>
+          <t>Sightlines</t>
         </is>
       </c>
       <c r="H19" s="24" t="inlineStr">
@@ -1561,7 +1571,7 @@
       </c>
       <c r="E20" s="25" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 12:00</t>
         </is>
       </c>
       <c r="F20" s="25" t="inlineStr">
@@ -1571,7 +1581,7 @@
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>Sliding and folding systems</t>
+          <t>Sliding and folding</t>
         </is>
       </c>
       <c r="H20" s="25" t="inlineStr">
@@ -1618,22 +1628,22 @@
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Educational</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>Stella, Sofia</t>
+          <t>Fixed vs operable</t>
         </is>
       </c>
       <c r="H21" s="16" t="inlineStr">
         <is>
-          <t>Photo + 2</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1673,7 +1683,11 @@
           <t>Mon</t>
         </is>
       </c>
-      <c r="E22" s="23" t="inlineStr"/>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t>9:00 (site)</t>
+        </is>
+      </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
           <t>(Website)</t>
@@ -1728,7 +1742,7 @@
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
@@ -1785,7 +1799,7 @@
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 18:00</t>
         </is>
       </c>
       <c r="F24" s="19" t="inlineStr">
@@ -1842,7 +1856,7 @@
       </c>
       <c r="E25" s="26" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F25" s="26" t="inlineStr">
@@ -1899,7 +1913,7 @@
       </c>
       <c r="E26" s="25" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F26" s="25" t="inlineStr">
@@ -1956,7 +1970,7 @@
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 18:00</t>
         </is>
       </c>
       <c r="F27" s="19" t="inlineStr">
@@ -2013,7 +2027,7 @@
       </c>
       <c r="E28" s="16" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F28" s="16" t="inlineStr">
@@ -2068,7 +2082,11 @@
           <t>Mon</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr"/>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>9:00 (site)</t>
+        </is>
+      </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
           <t>(Website)</t>
@@ -2123,7 +2141,7 @@
       </c>
       <c r="E30" s="18" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 / 12:00</t>
         </is>
       </c>
       <c r="F30" s="18" t="inlineStr">
@@ -2180,7 +2198,7 @@
       </c>
       <c r="E31" s="21" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>11:00 / 12:00</t>
         </is>
       </c>
       <c r="F31" s="21" t="inlineStr">
@@ -2237,7 +2255,7 @@
       </c>
       <c r="E32" s="26" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:00 / 11:00</t>
         </is>
       </c>
       <c r="F32" s="26" t="inlineStr">

</xml_diff>